<commit_message>
docs(hw3): reconcile verified issue mappings
</commit_message>
<xml_diff>
--- a/task1-gui/GUI_Checklist_HW3.xlsx
+++ b/task1-gui/GUI_Checklist_HW3.xlsx
@@ -2889,7 +2889,7 @@
       </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/45</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="R29" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/46</t>
         </is>
       </c>
     </row>
@@ -3073,7 +3073,7 @@
       </c>
       <c r="R30" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/46</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/45</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -6319,7 +6319,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/46</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/46</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs(hw3): publish remaining Task 1 issues
</commit_message>
<xml_diff>
--- a/task1-gui/GUI_Checklist_HW3.xlsx
+++ b/task1-gui/GUI_Checklist_HW3.xlsx
@@ -3837,7 +3837,7 @@
       </c>
       <c r="R39" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/291</t>
         </is>
       </c>
     </row>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="R41" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/292</t>
         </is>
       </c>
     </row>
@@ -4189,7 +4189,7 @@
       </c>
       <c r="R43" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/293</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="R44" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/294</t>
         </is>
       </c>
     </row>
@@ -4373,7 +4373,7 @@
       </c>
       <c r="R45" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/295</t>
         </is>
       </c>
     </row>
@@ -4633,7 +4633,7 @@
       </c>
       <c r="R48" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/296</t>
         </is>
       </c>
     </row>
@@ -4809,7 +4809,7 @@
       </c>
       <c r="R50" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/297</t>
         </is>
       </c>
     </row>
@@ -4985,7 +4985,7 @@
       </c>
       <c r="R52" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/297</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5497,7 @@
       </c>
       <c r="R58" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/298</t>
         </is>
       </c>
     </row>
@@ -6373,7 +6373,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/291</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -6400,7 +6400,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/292</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/293</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/294</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -6481,7 +6481,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/295</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/296</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/297</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/297</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -6589,7 +6589,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>PENDING_EXTERNAL_ACTION</t>
+          <t>https://github.com/trngnneee/eshop-sut/issues/298</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">

</xml_diff>